<commit_message>
Atualização da aplicação (desenvolvimento regional)
</commit_message>
<xml_diff>
--- a/dados/ICMS_Real.xlsx
+++ b/dados/ICMS_Real.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\guilh\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\victo\Documents\dev_2026\gd_impacta_mg\dados\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="8_{8ED8B095-6E97-4279-B18B-E1C2965344E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{2E1FBF1C-A30D-4840-B07A-61AAF03528DE}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="5" xr2:uid="{2E1FBF1C-A30D-4840-B07A-61AAF03528DE}"/>
   </bookViews>
   <sheets>
     <sheet name="ICMS" sheetId="1" r:id="rId1"/>
@@ -25,6 +25,17 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
   </extLst>
 </workbook>
 </file>
@@ -1044,7 +1055,7 @@
   <numFmts count="3">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="166" formatCode="_-* #,##0.0000_-;\-* #,##0.0000_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="165" formatCode="_-* #,##0.0000_-;\-* #,##0.0000_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="8" x14ac:knownFonts="1">
     <font>
@@ -1185,7 +1196,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
@@ -1206,9 +1217,8 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="43" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1229,9 +1239,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office 2013 - 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1269,7 +1279,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1375,7 +1385,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1517,7 +1527,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1526,20 +1536,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{05BC0CFD-EB6A-4ACE-B034-FD9F0E4714BB}">
   <dimension ref="A1:M128"/>
-  <sheetFormatPr defaultColWidth="12.109375" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="12.1328125" defaultRowHeight="13.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="15.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="66.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.77734375" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="12.109375" style="1"/>
-    <col min="6" max="6" width="19.21875" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.21875" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.21875" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="13" width="13.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="16384" width="12.109375" style="1"/>
+    <col min="1" max="1" width="15.1328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="66.86328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.796875" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="12.1328125" style="1"/>
+    <col min="6" max="6" width="19.19921875" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.19921875" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.19921875" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="13" width="13.53125" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="16384" width="12.1328125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" ht="13.9" x14ac:dyDescent="0.4">
       <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1547,7 +1557,7 @@
         <v>2023</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" ht="13.9" x14ac:dyDescent="0.4">
       <c r="B2" s="3" t="s">
         <v>1</v>
       </c>
@@ -1556,7 +1566,7 @@
         <v>51281981987</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A3" s="5" t="s">
         <v>2</v>
       </c>
@@ -1585,7 +1595,7 @@
       <c r="L3" s="7"/>
       <c r="M3" s="7"/>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="s">
         <v>4</v>
       </c>
@@ -1614,7 +1624,7 @@
       <c r="L4" s="7"/>
       <c r="M4" s="7"/>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A5" s="5" t="s">
         <v>7</v>
       </c>
@@ -1643,7 +1653,7 @@
       <c r="L5" s="7"/>
       <c r="M5" s="7"/>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A6" s="5" t="s">
         <v>9</v>
       </c>
@@ -1672,7 +1682,7 @@
       <c r="L6" s="7"/>
       <c r="M6" s="7"/>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A7" s="5" t="s">
         <v>11</v>
       </c>
@@ -1698,7 +1708,7 @@
       <c r="L7" s="7"/>
       <c r="M7" s="7"/>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A8" s="5" t="s">
         <v>13</v>
       </c>
@@ -1727,7 +1737,7 @@
       <c r="L8" s="7"/>
       <c r="M8" s="7"/>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A9" s="5" t="s">
         <v>15</v>
       </c>
@@ -1750,7 +1760,7 @@
       <c r="L9" s="7"/>
       <c r="M9" s="7"/>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A10" s="5" t="s">
         <v>16</v>
       </c>
@@ -1773,7 +1783,7 @@
       <c r="L10" s="7"/>
       <c r="M10" s="7"/>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A11" s="5" t="s">
         <v>18</v>
       </c>
@@ -1792,7 +1802,7 @@
       <c r="L11" s="7"/>
       <c r="M11" s="7"/>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A12" s="5" t="s">
         <v>20</v>
       </c>
@@ -1811,7 +1821,7 @@
       <c r="L12" s="7"/>
       <c r="M12" s="7"/>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A13" s="5" t="s">
         <v>22</v>
       </c>
@@ -1830,7 +1840,7 @@
       <c r="L13" s="7"/>
       <c r="M13" s="7"/>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A14" s="5" t="s">
         <v>24</v>
       </c>
@@ -1849,7 +1859,7 @@
       <c r="L14" s="7"/>
       <c r="M14" s="7"/>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A15" s="5" t="s">
         <v>26</v>
       </c>
@@ -1868,7 +1878,7 @@
       <c r="L15" s="7"/>
       <c r="M15" s="7"/>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A16" s="5" t="s">
         <v>28</v>
       </c>
@@ -1887,7 +1897,7 @@
       <c r="L16" s="7"/>
       <c r="M16" s="7"/>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A17" s="5" t="s">
         <v>30</v>
       </c>
@@ -1906,7 +1916,7 @@
       <c r="L17" s="7"/>
       <c r="M17" s="7"/>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A18" s="5" t="s">
         <v>32</v>
       </c>
@@ -1925,7 +1935,7 @@
       <c r="L18" s="7"/>
       <c r="M18" s="7"/>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A19" s="5" t="s">
         <v>34</v>
       </c>
@@ -1944,7 +1954,7 @@
       <c r="L19" s="7"/>
       <c r="M19" s="7"/>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A20" s="5" t="s">
         <v>36</v>
       </c>
@@ -1963,7 +1973,7 @@
       <c r="L20" s="7"/>
       <c r="M20" s="7"/>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A21" s="5" t="s">
         <v>38</v>
       </c>
@@ -1982,7 +1992,7 @@
       <c r="L21" s="7"/>
       <c r="M21" s="7"/>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A22" s="5" t="s">
         <v>40</v>
       </c>
@@ -2001,7 +2011,7 @@
       <c r="L22" s="7"/>
       <c r="M22" s="7"/>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A23" s="5" t="s">
         <v>42</v>
       </c>
@@ -2020,7 +2030,7 @@
       <c r="L23" s="7"/>
       <c r="M23" s="7"/>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A24" s="5" t="s">
         <v>44</v>
       </c>
@@ -2039,7 +2049,7 @@
       <c r="L24" s="7"/>
       <c r="M24" s="7"/>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A25" s="5" t="s">
         <v>46</v>
       </c>
@@ -2058,7 +2068,7 @@
       <c r="L25" s="7"/>
       <c r="M25" s="7"/>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A26" s="5" t="s">
         <v>48</v>
       </c>
@@ -2077,7 +2087,7 @@
       <c r="L26" s="7"/>
       <c r="M26" s="7"/>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A27" s="5" t="s">
         <v>50</v>
       </c>
@@ -2096,7 +2106,7 @@
       <c r="L27" s="7"/>
       <c r="M27" s="7"/>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A28" s="5" t="s">
         <v>52</v>
       </c>
@@ -2115,7 +2125,7 @@
       <c r="L28" s="7"/>
       <c r="M28" s="7"/>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A29" s="5" t="s">
         <v>54</v>
       </c>
@@ -2134,7 +2144,7 @@
       <c r="L29" s="7"/>
       <c r="M29" s="7"/>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A30" s="5" t="s">
         <v>56</v>
       </c>
@@ -2153,7 +2163,7 @@
       <c r="L30" s="7"/>
       <c r="M30" s="7"/>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A31" s="5" t="s">
         <v>58</v>
       </c>
@@ -2172,7 +2182,7 @@
       <c r="L31" s="7"/>
       <c r="M31" s="7"/>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A32" s="5" t="s">
         <v>60</v>
       </c>
@@ -2191,7 +2201,7 @@
       <c r="L32" s="7"/>
       <c r="M32" s="7"/>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A33" s="5" t="s">
         <v>62</v>
       </c>
@@ -2210,7 +2220,7 @@
       <c r="L33" s="7"/>
       <c r="M33" s="7"/>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A34" s="5" t="s">
         <v>64</v>
       </c>
@@ -2229,7 +2239,7 @@
       <c r="L34" s="7"/>
       <c r="M34" s="7"/>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A35" s="5" t="s">
         <v>66</v>
       </c>
@@ -2248,7 +2258,7 @@
       <c r="L35" s="7"/>
       <c r="M35" s="7"/>
     </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A36" s="5" t="s">
         <v>68</v>
       </c>
@@ -2267,7 +2277,7 @@
       <c r="L36" s="7"/>
       <c r="M36" s="7"/>
     </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A37" s="5" t="s">
         <v>70</v>
       </c>
@@ -2286,7 +2296,7 @@
       <c r="L37" s="7"/>
       <c r="M37" s="7"/>
     </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A38" s="5" t="s">
         <v>71</v>
       </c>
@@ -2305,7 +2315,7 @@
       <c r="L38" s="7"/>
       <c r="M38" s="7"/>
     </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A39" s="5" t="s">
         <v>73</v>
       </c>
@@ -2324,7 +2334,7 @@
       <c r="L39" s="7"/>
       <c r="M39" s="7"/>
     </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A40" s="5" t="s">
         <v>75</v>
       </c>
@@ -2343,7 +2353,7 @@
       <c r="L40" s="7"/>
       <c r="M40" s="7"/>
     </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A41" s="5" t="s">
         <v>76</v>
       </c>
@@ -2362,7 +2372,7 @@
       <c r="L41" s="7"/>
       <c r="M41" s="7"/>
     </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A42" s="5" t="s">
         <v>78</v>
       </c>
@@ -2381,7 +2391,7 @@
       <c r="L42" s="7"/>
       <c r="M42" s="7"/>
     </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A43" s="5" t="s">
         <v>80</v>
       </c>
@@ -2400,7 +2410,7 @@
       <c r="L43" s="7"/>
       <c r="M43" s="7"/>
     </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A44" s="5" t="s">
         <v>82</v>
       </c>
@@ -2419,7 +2429,7 @@
       <c r="L44" s="7"/>
       <c r="M44" s="7"/>
     </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A45" s="5" t="s">
         <v>84</v>
       </c>
@@ -2438,7 +2448,7 @@
       <c r="L45" s="7"/>
       <c r="M45" s="7"/>
     </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A46" s="5" t="s">
         <v>85</v>
       </c>
@@ -2457,7 +2467,7 @@
       <c r="L46" s="7"/>
       <c r="M46" s="7"/>
     </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A47" s="5" t="s">
         <v>87</v>
       </c>
@@ -2476,7 +2486,7 @@
       <c r="L47" s="7"/>
       <c r="M47" s="7"/>
     </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A48" s="5" t="s">
         <v>89</v>
       </c>
@@ -2495,7 +2505,7 @@
       <c r="L48" s="7"/>
       <c r="M48" s="7"/>
     </row>
-    <row r="49" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A49" s="5" t="s">
         <v>91</v>
       </c>
@@ -2514,7 +2524,7 @@
       <c r="L49" s="7"/>
       <c r="M49" s="7"/>
     </row>
-    <row r="50" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A50" s="5" t="s">
         <v>93</v>
       </c>
@@ -2533,7 +2543,7 @@
       <c r="L50" s="7"/>
       <c r="M50" s="7"/>
     </row>
-    <row r="51" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A51" s="5" t="s">
         <v>95</v>
       </c>
@@ -2552,7 +2562,7 @@
       <c r="L51" s="7"/>
       <c r="M51" s="7"/>
     </row>
-    <row r="52" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A52" s="5" t="s">
         <v>97</v>
       </c>
@@ -2571,7 +2581,7 @@
       <c r="L52" s="7"/>
       <c r="M52" s="7"/>
     </row>
-    <row r="53" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A53" s="5" t="s">
         <v>99</v>
       </c>
@@ -2590,7 +2600,7 @@
       <c r="L53" s="7"/>
       <c r="M53" s="7"/>
     </row>
-    <row r="54" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A54" s="5" t="s">
         <v>101</v>
       </c>
@@ -2609,7 +2619,7 @@
       <c r="L54" s="7"/>
       <c r="M54" s="7"/>
     </row>
-    <row r="55" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A55" s="5" t="s">
         <v>103</v>
       </c>
@@ -2628,7 +2638,7 @@
       <c r="L55" s="7"/>
       <c r="M55" s="7"/>
     </row>
-    <row r="56" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A56" s="5" t="s">
         <v>105</v>
       </c>
@@ -2647,7 +2657,7 @@
       <c r="L56" s="7"/>
       <c r="M56" s="7"/>
     </row>
-    <row r="57" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A57" s="5" t="s">
         <v>107</v>
       </c>
@@ -2666,7 +2676,7 @@
       <c r="L57" s="7"/>
       <c r="M57" s="7"/>
     </row>
-    <row r="58" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A58" s="5" t="s">
         <v>109</v>
       </c>
@@ -2685,7 +2695,7 @@
       <c r="L58" s="7"/>
       <c r="M58" s="7"/>
     </row>
-    <row r="59" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A59" s="5" t="s">
         <v>111</v>
       </c>
@@ -2704,7 +2714,7 @@
       <c r="L59" s="7"/>
       <c r="M59" s="7"/>
     </row>
-    <row r="60" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A60" s="5" t="s">
         <v>113</v>
       </c>
@@ -2723,7 +2733,7 @@
       <c r="L60" s="7"/>
       <c r="M60" s="7"/>
     </row>
-    <row r="61" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A61" s="5" t="s">
         <v>115</v>
       </c>
@@ -2742,7 +2752,7 @@
       <c r="L61" s="7"/>
       <c r="M61" s="7"/>
     </row>
-    <row r="62" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A62" s="5" t="s">
         <v>117</v>
       </c>
@@ -2761,7 +2771,7 @@
       <c r="L62" s="7"/>
       <c r="M62" s="7"/>
     </row>
-    <row r="63" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A63" s="5" t="s">
         <v>119</v>
       </c>
@@ -2780,7 +2790,7 @@
       <c r="L63" s="7"/>
       <c r="M63" s="7"/>
     </row>
-    <row r="64" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A64" s="5" t="s">
         <v>121</v>
       </c>
@@ -2799,7 +2809,7 @@
       <c r="L64" s="7"/>
       <c r="M64" s="7"/>
     </row>
-    <row r="65" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A65" s="5" t="s">
         <v>123</v>
       </c>
@@ -2818,7 +2828,7 @@
       <c r="L65" s="7"/>
       <c r="M65" s="7"/>
     </row>
-    <row r="66" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A66" s="5" t="s">
         <v>125</v>
       </c>
@@ -2829,7 +2839,7 @@
         <v>833041316</v>
       </c>
     </row>
-    <row r="67" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A67" s="5" t="s">
         <v>126</v>
       </c>
@@ -2840,7 +2850,7 @@
         <v>125348802</v>
       </c>
     </row>
-    <row r="68" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A68" s="5" t="s">
         <v>128</v>
       </c>
@@ -2851,7 +2861,7 @@
         <v>435930727</v>
       </c>
     </row>
-    <row r="69" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A69" s="5" t="s">
         <v>130</v>
       </c>
@@ -2862,7 +2872,7 @@
         <v>143724190</v>
       </c>
     </row>
-    <row r="70" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A70" s="5" t="s">
         <v>132</v>
       </c>
@@ -2873,7 +2883,7 @@
         <v>1526093799</v>
       </c>
     </row>
-    <row r="71" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A71" s="5" t="s">
         <v>134</v>
       </c>
@@ -2884,7 +2894,7 @@
         <v>118787448</v>
       </c>
     </row>
-    <row r="72" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A72" s="5" t="s">
         <v>136</v>
       </c>
@@ -2895,7 +2905,7 @@
         <v>195112464</v>
       </c>
     </row>
-    <row r="73" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A73" s="5" t="s">
         <v>138</v>
       </c>
@@ -2906,7 +2916,7 @@
         <v>866703289</v>
       </c>
     </row>
-    <row r="74" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A74" s="5" t="s">
         <v>140</v>
       </c>
@@ -2917,7 +2927,7 @@
         <v>19640818</v>
       </c>
     </row>
-    <row r="75" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A75" s="5" t="s">
         <v>142</v>
       </c>
@@ -2928,7 +2938,7 @@
         <v>116935703</v>
       </c>
     </row>
-    <row r="76" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A76" s="5" t="s">
         <v>144</v>
       </c>
@@ -2939,7 +2949,7 @@
         <v>15590918</v>
       </c>
     </row>
-    <row r="77" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A77" s="5" t="s">
         <v>146</v>
       </c>
@@ -2950,7 +2960,7 @@
         <v>152254724</v>
       </c>
     </row>
-    <row r="78" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A78" s="5" t="s">
         <v>148</v>
       </c>
@@ -2961,7 +2971,7 @@
         <v>292347379</v>
       </c>
     </row>
-    <row r="79" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A79" s="5" t="s">
         <v>150</v>
       </c>
@@ -2972,7 +2982,7 @@
         <v>65190189</v>
       </c>
     </row>
-    <row r="80" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A80" s="5" t="s">
         <v>152</v>
       </c>
@@ -2983,7 +2993,7 @@
         <v>45559054</v>
       </c>
     </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A81" s="5" t="s">
         <v>154</v>
       </c>
@@ -2994,7 +3004,7 @@
         <v>209078433</v>
       </c>
     </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A82" s="5" t="s">
         <v>156</v>
       </c>
@@ -3005,7 +3015,7 @@
         <v>252186325</v>
       </c>
     </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A83" s="5" t="s">
         <v>158</v>
       </c>
@@ -3016,7 +3026,7 @@
         <v>737432020</v>
       </c>
     </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A84" s="5" t="s">
         <v>160</v>
       </c>
@@ -3027,7 +3037,7 @@
         <v>168958200</v>
       </c>
     </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A85" s="5" t="s">
         <v>162</v>
       </c>
@@ -3038,7 +3048,7 @@
         <v>495605489</v>
       </c>
     </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A86" s="5" t="s">
         <v>164</v>
       </c>
@@ -3049,7 +3059,7 @@
         <v>55538538</v>
       </c>
     </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A87" s="5" t="s">
         <v>166</v>
       </c>
@@ -3060,7 +3070,7 @@
         <v>237347664</v>
       </c>
     </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A88" s="5" t="s">
         <v>168</v>
       </c>
@@ -3071,7 +3081,7 @@
         <v>58083898</v>
       </c>
     </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A89" s="5" t="s">
         <v>170</v>
       </c>
@@ -3082,7 +3092,7 @@
         <v>88323711</v>
       </c>
     </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A90" s="5" t="s">
         <v>172</v>
       </c>
@@ -3093,7 +3103,7 @@
         <v>4934225117</v>
       </c>
     </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A91" s="5" t="s">
         <v>174</v>
       </c>
@@ -3104,7 +3114,7 @@
         <v>71546706</v>
       </c>
     </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A92" s="5" t="s">
         <v>176</v>
       </c>
@@ -3115,7 +3125,7 @@
         <v>14400917</v>
       </c>
     </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A93" s="5" t="s">
         <v>178</v>
       </c>
@@ -3126,7 +3136,7 @@
         <v>6317429</v>
       </c>
     </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A94" s="5" t="s">
         <v>180</v>
       </c>
@@ -3137,7 +3147,7 @@
         <v>27699461</v>
       </c>
     </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A95" s="5" t="s">
         <v>182</v>
       </c>
@@ -3148,7 +3158,7 @@
         <v>16495663209</v>
       </c>
     </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A96" s="5" t="s">
         <v>184</v>
       </c>
@@ -3159,7 +3169,7 @@
         <v>816275243</v>
       </c>
     </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A97" s="5" t="s">
         <v>186</v>
       </c>
@@ -3170,7 +3180,7 @@
         <v>214224642</v>
       </c>
     </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A98" s="5" t="s">
         <v>188</v>
       </c>
@@ -3181,7 +3191,7 @@
         <v>5127669</v>
       </c>
     </row>
-    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A99" s="5" t="s">
         <v>190</v>
       </c>
@@ -3192,7 +3202,7 @@
         <v>48967808</v>
       </c>
     </row>
-    <row r="100" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A100" s="5" t="s">
         <v>192</v>
       </c>
@@ -3203,7 +3213,7 @@
         <v>4994968</v>
       </c>
     </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A101" s="5" t="s">
         <v>194</v>
       </c>
@@ -3214,7 +3224,7 @@
         <v>12635896</v>
       </c>
     </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A102" s="5" t="s">
         <v>196</v>
       </c>
@@ -3225,7 +3235,7 @@
         <v>228444430</v>
       </c>
     </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A103" s="5" t="s">
         <v>198</v>
       </c>
@@ -3236,7 +3246,7 @@
         <v>839601</v>
       </c>
     </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A104" s="5" t="s">
         <v>200</v>
       </c>
@@ -3247,7 +3257,7 @@
         <v>13227674</v>
       </c>
     </row>
-    <row r="105" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A105" s="5" t="s">
         <v>202</v>
       </c>
@@ -3258,7 +3268,7 @@
         <v>1741023533</v>
       </c>
     </row>
-    <row r="106" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A106" s="5" t="s">
         <v>204</v>
       </c>
@@ -3269,7 +3279,7 @@
         <v>24500364</v>
       </c>
     </row>
-    <row r="107" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A107" s="5" t="s">
         <v>206</v>
       </c>
@@ -3280,7 +3290,7 @@
         <v>669072</v>
       </c>
     </row>
-    <row r="108" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A108" s="5" t="s">
         <v>208</v>
       </c>
@@ -3291,7 +3301,7 @@
         <v>1231670</v>
       </c>
     </row>
-    <row r="109" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A109" s="5" t="s">
         <v>210</v>
       </c>
@@ -3302,7 +3312,7 @@
         <v>8858</v>
       </c>
     </row>
-    <row r="110" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A110" s="5" t="s">
         <v>212</v>
       </c>
@@ -3313,7 +3323,7 @@
         <v>1597958</v>
       </c>
     </row>
-    <row r="111" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A111" s="5" t="s">
         <v>214</v>
       </c>
@@ -3324,7 +3334,7 @@
         <v>9235842</v>
       </c>
     </row>
-    <row r="112" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A112" s="5" t="s">
         <v>216</v>
       </c>
@@ -3335,7 +3345,7 @@
         <v>8863256</v>
       </c>
     </row>
-    <row r="113" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A113" s="5" t="s">
         <v>218</v>
       </c>
@@ -3346,7 +3356,7 @@
         <v>73695524</v>
       </c>
     </row>
-    <row r="114" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A114" s="5" t="s">
         <v>220</v>
       </c>
@@ -3357,7 +3367,7 @@
         <v>27947537</v>
       </c>
     </row>
-    <row r="115" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A115" s="5" t="s">
         <v>222</v>
       </c>
@@ -3368,7 +3378,7 @@
         <v>24113</v>
       </c>
     </row>
-    <row r="116" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A116" s="5" t="s">
         <v>224</v>
       </c>
@@ -3379,7 +3389,7 @@
         <v>49317713</v>
       </c>
     </row>
-    <row r="117" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A117" s="5" t="s">
         <v>226</v>
       </c>
@@ -3390,7 +3400,7 @@
         <v>36314088</v>
       </c>
     </row>
-    <row r="118" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A118" s="5" t="s">
         <v>228</v>
       </c>
@@ -3401,7 +3411,7 @@
         <v>279538</v>
       </c>
     </row>
-    <row r="119" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A119" s="5" t="s">
         <v>230</v>
       </c>
@@ -3412,7 +3422,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="120" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A120" s="5" t="s">
         <v>232</v>
       </c>
@@ -3423,7 +3433,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="121" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A121" s="5" t="s">
         <v>234</v>
       </c>
@@ -3434,7 +3444,7 @@
         <v>7529884</v>
       </c>
     </row>
-    <row r="122" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A122" s="5" t="s">
         <v>236</v>
       </c>
@@ -3445,7 +3455,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="123" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A123" s="5" t="s">
         <v>238</v>
       </c>
@@ -3456,7 +3466,7 @@
         <v>532309</v>
       </c>
     </row>
-    <row r="124" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A124" s="5" t="s">
         <v>240</v>
       </c>
@@ -3467,7 +3477,7 @@
         <v>5714492</v>
       </c>
     </row>
-    <row r="125" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A125" s="5" t="s">
         <v>242</v>
       </c>
@@ -3478,7 +3488,7 @@
         <v>5847786</v>
       </c>
     </row>
-    <row r="126" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A126" s="5" t="s">
         <v>244</v>
       </c>
@@ -3489,7 +3499,7 @@
         <v>5086235</v>
       </c>
     </row>
-    <row r="127" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A127" s="5" t="s">
         <v>246</v>
       </c>
@@ -3500,7 +3510,7 @@
         <v>519504</v>
       </c>
     </row>
-    <row r="128" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A128" s="5" t="s">
         <v>248</v>
       </c>
@@ -3519,12 +3529,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8609ED16-5AED-4AA1-8C02-B38D89259A6D}">
   <dimension ref="A1:BP7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.53125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:68" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>329</v>
       </c>
@@ -3730,7 +3740,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="2" spans="1:68" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>323</v>
       </c>
@@ -3936,7 +3946,7 @@
         <v>2.5110000000000001</v>
       </c>
     </row>
-    <row r="3" spans="1:68" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>324</v>
       </c>
@@ -4142,7 +4152,7 @@
         <v>1.083</v>
       </c>
     </row>
-    <row r="4" spans="1:68" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>325</v>
       </c>
@@ -4348,7 +4358,7 @@
         <v>1.78</v>
       </c>
     </row>
-    <row r="5" spans="1:68" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>326</v>
       </c>
@@ -4554,7 +4564,7 @@
         <v>0.55800000000000005</v>
       </c>
     </row>
-    <row r="6" spans="1:68" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>327</v>
       </c>
@@ -4760,7 +4770,7 @@
         <v>1.1930000000000001</v>
       </c>
     </row>
-    <row r="7" spans="1:68" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>328</v>
       </c>
@@ -4974,13 +4984,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20FBF4F2-6712-4BE0-AC39-1737866AEEBA}">
   <dimension ref="A1:BP10"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="12.5546875" bestFit="1" customWidth="1"/>
-    <col min="68" max="68" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.53125" bestFit="1" customWidth="1"/>
+    <col min="68" max="68" width="11.46484375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:68" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>332</v>
       </c>
@@ -5186,7 +5196,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="2" spans="1:68" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>323</v>
       </c>
@@ -5393,7 +5403,7 @@
         <v>75381.023000000001</v>
       </c>
     </row>
-    <row r="3" spans="1:68" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>324</v>
       </c>
@@ -5600,7 +5610,7 @@
         <v>23572.288999999986</v>
       </c>
     </row>
-    <row r="4" spans="1:68" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>325</v>
       </c>
@@ -5807,7 +5817,7 @@
         <v>234961.79599999989</v>
       </c>
     </row>
-    <row r="5" spans="1:68" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>330</v>
       </c>
@@ -6014,7 +6024,7 @@
         <v>7295.2570000000042</v>
       </c>
     </row>
-    <row r="6" spans="1:68" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>331</v>
       </c>
@@ -6221,7 +6231,7 @@
         <v>15300.126000000002</v>
       </c>
     </row>
-    <row r="7" spans="1:68" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>326</v>
       </c>
@@ -6428,7 +6438,7 @@
         <v>426918.35600000003</v>
       </c>
     </row>
-    <row r="8" spans="1:68" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>327</v>
       </c>
@@ -6635,7 +6645,7 @@
         <v>78888.088999999993</v>
       </c>
     </row>
-    <row r="9" spans="1:68" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>328</v>
       </c>
@@ -6842,7 +6852,7 @@
         <v>23856.275000000009</v>
       </c>
     </row>
-    <row r="10" spans="1:68" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A10" s="17" t="s">
         <v>333</v>
       </c>
@@ -7119,13 +7129,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20E20087-E8E5-40BE-9FB5-6F2CD4499898}">
   <dimension ref="A1:BP10"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="12.5546875" bestFit="1" customWidth="1"/>
-    <col min="68" max="68" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.53125" bestFit="1" customWidth="1"/>
+    <col min="68" max="68" width="11.46484375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:68" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>332</v>
       </c>
@@ -7331,7 +7341,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="2" spans="1:68" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>323</v>
       </c>
@@ -7604,7 +7614,7 @@
         <v>0.99999999999999967</v>
       </c>
     </row>
-    <row r="3" spans="1:68" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>324</v>
       </c>
@@ -7877,7 +7887,7 @@
         <v>1.0000000000000007</v>
       </c>
     </row>
-    <row r="4" spans="1:68" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>325</v>
       </c>
@@ -8150,7 +8160,7 @@
         <v>1.0000000000000004</v>
       </c>
     </row>
-    <row r="5" spans="1:68" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>330</v>
       </c>
@@ -8423,7 +8433,7 @@
         <v>0.99999999999999933</v>
       </c>
     </row>
-    <row r="6" spans="1:68" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>331</v>
       </c>
@@ -8696,7 +8706,7 @@
         <v>0.99999999999999989</v>
       </c>
     </row>
-    <row r="7" spans="1:68" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>326</v>
       </c>
@@ -8969,7 +8979,7 @@
         <v>0.99999999999999989</v>
       </c>
     </row>
-    <row r="8" spans="1:68" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>327</v>
       </c>
@@ -9242,7 +9252,7 @@
         <v>1.0000000000000002</v>
       </c>
     </row>
-    <row r="9" spans="1:68" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>328</v>
       </c>
@@ -9515,7 +9525,7 @@
         <v>0.99999999999999956</v>
       </c>
     </row>
-    <row r="10" spans="1:68" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A10" s="17"/>
       <c r="B10" s="17"/>
       <c r="C10" s="17"/>
@@ -9592,47 +9602,47 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ADAA92CA-8B6F-4507-823B-B0B2D73235FC}">
   <dimension ref="A1:BP8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="12.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="6" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="16.88671875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.44140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="16.88671875" bestFit="1" customWidth="1"/>
-    <col min="12" max="14" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="16.88671875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="16.88671875" bestFit="1" customWidth="1"/>
-    <col min="18" max="19" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="20" max="23" width="16.88671875" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="26" max="27" width="18.44140625" bestFit="1" customWidth="1"/>
-    <col min="28" max="30" width="16.88671875" bestFit="1" customWidth="1"/>
-    <col min="31" max="32" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="33" max="35" width="16.88671875" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="37" max="38" width="16.88671875" bestFit="1" customWidth="1"/>
-    <col min="39" max="40" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="18.44140625" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="43" max="46" width="16.88671875" bestFit="1" customWidth="1"/>
-    <col min="47" max="48" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="16.88671875" bestFit="1" customWidth="1"/>
-    <col min="50" max="50" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="51" max="51" width="16.88671875" bestFit="1" customWidth="1"/>
-    <col min="52" max="52" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="16.88671875" bestFit="1" customWidth="1"/>
-    <col min="54" max="54" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="55" max="63" width="16.88671875" bestFit="1" customWidth="1"/>
-    <col min="64" max="64" width="18.44140625" bestFit="1" customWidth="1"/>
-    <col min="65" max="66" width="16.88671875" bestFit="1" customWidth="1"/>
-    <col min="67" max="67" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="68" max="68" width="17.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.53125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.86328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.86328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="6" width="15.86328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="16.86328125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.46484375" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="16.86328125" bestFit="1" customWidth="1"/>
+    <col min="12" max="14" width="15.86328125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="16.86328125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="15.86328125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="16.86328125" bestFit="1" customWidth="1"/>
+    <col min="18" max="19" width="15.86328125" bestFit="1" customWidth="1"/>
+    <col min="20" max="23" width="16.86328125" bestFit="1" customWidth="1"/>
+    <col min="24" max="25" width="15.86328125" bestFit="1" customWidth="1"/>
+    <col min="26" max="27" width="18.46484375" bestFit="1" customWidth="1"/>
+    <col min="28" max="30" width="16.86328125" bestFit="1" customWidth="1"/>
+    <col min="31" max="32" width="15.86328125" bestFit="1" customWidth="1"/>
+    <col min="33" max="35" width="16.86328125" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="15.86328125" bestFit="1" customWidth="1"/>
+    <col min="37" max="38" width="16.86328125" bestFit="1" customWidth="1"/>
+    <col min="39" max="40" width="15.86328125" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="18.46484375" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="15.86328125" bestFit="1" customWidth="1"/>
+    <col min="43" max="46" width="16.86328125" bestFit="1" customWidth="1"/>
+    <col min="47" max="48" width="15.86328125" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="16.86328125" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="15.86328125" bestFit="1" customWidth="1"/>
+    <col min="51" max="51" width="16.86328125" bestFit="1" customWidth="1"/>
+    <col min="52" max="52" width="15.86328125" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="16.86328125" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="15.86328125" bestFit="1" customWidth="1"/>
+    <col min="55" max="63" width="16.86328125" bestFit="1" customWidth="1"/>
+    <col min="64" max="64" width="18.46484375" bestFit="1" customWidth="1"/>
+    <col min="65" max="66" width="16.86328125" bestFit="1" customWidth="1"/>
+    <col min="67" max="67" width="15.86328125" bestFit="1" customWidth="1"/>
+    <col min="68" max="68" width="17.796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:68" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>332</v>
       </c>
@@ -9838,7 +9848,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="2" spans="1:68" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>323</v>
       </c>
@@ -10111,7 +10121,7 @@
         <v>443411827</v>
       </c>
     </row>
-    <row r="3" spans="1:68" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>324</v>
       </c>
@@ -10384,7 +10394,7 @@
         <v>1712736919.0000014</v>
       </c>
     </row>
-    <row r="4" spans="1:68" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>325</v>
       </c>
@@ -10657,7 +10667,7 @@
         <v>24231303195.000019</v>
       </c>
     </row>
-    <row r="5" spans="1:68" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>326</v>
       </c>
@@ -10930,7 +10940,7 @@
         <v>2648366477</v>
       </c>
     </row>
-    <row r="6" spans="1:68" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>327</v>
       </c>
@@ -11203,7 +11213,7 @@
         <v>16495663209.000004</v>
       </c>
     </row>
-    <row r="7" spans="1:68" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>328</v>
       </c>
@@ -11476,7 +11486,7 @@
         <v>816275243</v>
       </c>
     </row>
-    <row r="8" spans="1:68" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A8" s="17"/>
       <c r="B8" s="17"/>
       <c r="C8" s="17"/>
@@ -11553,51 +11563,51 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF66A185-4EC7-402F-984B-24294ACFB5F9}">
   <dimension ref="A1:BP9"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.53125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="17" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.53125" bestFit="1" customWidth="1"/>
     <col min="4" max="6" width="17" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.53125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="17" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19.5546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.53125" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="18.53125" bestFit="1" customWidth="1"/>
     <col min="12" max="16" width="17" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="18.53125" bestFit="1" customWidth="1"/>
     <col min="18" max="19" width="17" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="18.53125" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="17" bestFit="1" customWidth="1"/>
-    <col min="22" max="23" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="22" max="23" width="18.53125" bestFit="1" customWidth="1"/>
     <col min="24" max="25" width="17" bestFit="1" customWidth="1"/>
-    <col min="26" max="28" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="26" max="28" width="18.53125" bestFit="1" customWidth="1"/>
     <col min="29" max="32" width="17" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="18.53125" bestFit="1" customWidth="1"/>
     <col min="34" max="34" width="17" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="18.53125" bestFit="1" customWidth="1"/>
     <col min="36" max="36" width="17" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="18.53125" bestFit="1" customWidth="1"/>
     <col min="38" max="40" width="17" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="18.53125" bestFit="1" customWidth="1"/>
     <col min="42" max="43" width="17" bestFit="1" customWidth="1"/>
-    <col min="44" max="46" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="44" max="46" width="18.53125" bestFit="1" customWidth="1"/>
     <col min="47" max="48" width="17" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="18.53125" bestFit="1" customWidth="1"/>
     <col min="50" max="50" width="17" bestFit="1" customWidth="1"/>
-    <col min="51" max="51" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="51" max="51" width="18.53125" bestFit="1" customWidth="1"/>
     <col min="52" max="52" width="17" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="18.53125" bestFit="1" customWidth="1"/>
     <col min="54" max="57" width="17" bestFit="1" customWidth="1"/>
-    <col min="58" max="59" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="58" max="59" width="18.53125" bestFit="1" customWidth="1"/>
     <col min="60" max="60" width="17" bestFit="1" customWidth="1"/>
-    <col min="61" max="64" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="61" max="64" width="18.53125" bestFit="1" customWidth="1"/>
     <col min="65" max="65" width="17" bestFit="1" customWidth="1"/>
-    <col min="66" max="66" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="66" max="66" width="18.53125" bestFit="1" customWidth="1"/>
     <col min="67" max="67" width="17" bestFit="1" customWidth="1"/>
-    <col min="68" max="68" width="19.77734375" bestFit="1" customWidth="1"/>
+    <col min="68" max="68" width="19.796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:68" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>332</v>
       </c>
@@ -11803,7 +11813,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="2" spans="1:68" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>323</v>
       </c>
@@ -12071,12 +12081,12 @@
         <f t="array" ref="BO2">ICMS_Micro!BO2*xtot!BO2</f>
         <v>30060079.564734828</v>
       </c>
-      <c r="BP2" s="22">
+      <c r="BP2" s="18">
         <f t="array" ref="BP2">SUM(B2:BO2)</f>
         <v>1641845506.0380931</v>
       </c>
     </row>
-    <row r="3" spans="1:68" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>324</v>
       </c>
@@ -12344,12 +12354,12 @@
         <f t="array" ref="BO3">ICMS_Micro!BO3*xtot!BO3</f>
         <v>8617322.5678500962</v>
       </c>
-      <c r="BP3" s="22">
+      <c r="BP3" s="18">
         <f t="array" ref="BP3">SUM(B3:BO3)</f>
         <v>9793993673.4852333</v>
       </c>
     </row>
-    <row r="4" spans="1:68" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>325</v>
       </c>
@@ -12617,12 +12627,12 @@
         <f t="array" ref="BO4">ICMS_Micro!BO4*xtot!BO4</f>
         <v>238252099.53451517</v>
       </c>
-      <c r="BP4" s="22">
+      <c r="BP4" s="18">
         <f t="array" ref="BP4">SUM(B4:BO4)</f>
         <v>109614117808.27655</v>
       </c>
     </row>
-    <row r="5" spans="1:68" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>326</v>
       </c>
@@ -12890,12 +12900,12 @@
         <f t="array" ref="BO5">ICMS_Micro!BO5*xtot!BO5</f>
         <v>30966489.797677282</v>
       </c>
-      <c r="BP5" s="22">
+      <c r="BP5" s="18">
         <f t="array" ref="BP5">SUM(B5:BO5)</f>
         <v>8471463297.567687</v>
       </c>
     </row>
-    <row r="6" spans="1:68" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>327</v>
       </c>
@@ -13163,12 +13173,12 @@
         <f t="array" ref="BO6">ICMS_Micro!BO6*xtot!BO6</f>
         <v>652684933.83039403</v>
       </c>
-      <c r="BP6" s="22">
+      <c r="BP6" s="18">
         <f t="array" ref="BP6">SUM(B6:BO6)</f>
         <v>95431921069.94783</v>
       </c>
     </row>
-    <row r="7" spans="1:68" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>328</v>
       </c>
@@ -13436,12 +13446,12 @@
         <f t="array" ref="BO7">ICMS_Micro!BO7*xtot!BO7</f>
         <v>12218658.591610068</v>
       </c>
-      <c r="BP7" s="22">
+      <c r="BP7" s="18">
         <f t="array" ref="BP7">SUM(B7:BO7)</f>
         <v>1895781760.2001584</v>
       </c>
     </row>
-    <row r="9" spans="1:68" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:68" x14ac:dyDescent="0.45">
       <c r="BP9" s="21">
         <f t="array" ref="BP9">SUM(BP2:BP7)</f>
         <v>226849123115.51556</v>

</xml_diff>